<commit_message>
Update reports 2026-10-06 10:07
</commit_message>
<xml_diff>
--- a/gex_pivot_levels_2026-10-06.xlsx
+++ b/gex_pivot_levels_2026-10-06.xlsx
@@ -544,12 +544,12 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>-$3.16M</t>
+          <t>-$3.05M</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>+$10.71M</t>
+          <t>+$10.83M</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -602,12 +602,12 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>-$5.30M</t>
+          <t>-$5.41M</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>+$12.87M</t>
+          <t>+$13.14M</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -664,12 +664,12 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>-$2.31M</t>
+          <t>-$2.35M</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>+$21.18M</t>
+          <t>+$21.52M</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -726,12 +726,12 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>-$1.84M</t>
+          <t>-$1.89M</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>+$19.05M</t>
+          <t>+$19.55M</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -755,12 +755,12 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>+$7.18M</t>
+          <t>+$7.32M</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>+$32.70M</t>
+          <t>+$33.37M</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -817,12 +817,12 @@
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>+$25.66M</t>
+          <t>+$26.15M</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>+$46.61M</t>
+          <t>+$47.50M</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
@@ -945,12 +945,12 @@
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>+$8.40M</t>
+          <t>+$7.73M</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>+$8.49M</t>
+          <t>+$7.81M</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
@@ -978,12 +978,12 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>+$16.43M</t>
+          <t>+$14.55M</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>+$16.47M</t>
+          <t>+$14.59M</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
@@ -1007,12 +1007,12 @@
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>+$19.71M</t>
+          <t>+$15.77M</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>+$19.78M</t>
+          <t>+$15.83M</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
@@ -1040,12 +1040,12 @@
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>+$6.55M</t>
+          <t>+$5.36M</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>+$6.56M</t>
+          <t>+$5.37M</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
@@ -3005,12 +3005,12 @@
       </c>
       <c r="E2" s="9" t="inlineStr">
         <is>
-          <t>+$25.66M</t>
+          <t>+$26.15M</t>
         </is>
       </c>
       <c r="F2" s="7" t="inlineStr">
         <is>
-          <t>+$46.61M</t>
+          <t>+$47.50M</t>
         </is>
       </c>
       <c r="G2" s="7" t="inlineStr">
@@ -3119,12 +3119,12 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>+$7.18M</t>
+          <t>+$7.32M</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>+$32.70M</t>
+          <t>+$33.37M</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -3153,12 +3153,12 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>-$2.31M</t>
+          <t>-$2.35M</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>+$21.18M</t>
+          <t>+$21.52M</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -3241,40 +3241,40 @@
       <c r="H8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B9" s="6" t="n">
-        <v>7919.55</v>
-      </c>
-      <c r="C9" s="6" t="n">
-        <v>7860</v>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="B9" s="2" t="n">
+        <v>7864.55</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>7805</v>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
-        <is>
-          <t>+$19.71M</t>
-        </is>
-      </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>+$19.78M</t>
-        </is>
-      </c>
-      <c r="G9" s="7" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H9" s="7" t="inlineStr">
-        <is>
-          <t>peak</t>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>+$17.83M</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>+$19.62M</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
         </is>
       </c>
     </row>
@@ -3285,36 +3285,32 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>7864.55</v>
+        <v>7819.55</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>7805</v>
+        <v>7760</v>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>+$17.83M</t>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>-$1.89M</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>+$19.62M</t>
+          <t>+$19.55M</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H10" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -3323,168 +3319,172 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>7819.55</v>
+        <v>7805.11</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>7760</v>
+        <v>772</v>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>+$7.54M</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>+$17.71M</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n">
+        <v>7919.55</v>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>7860</v>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>-$1.84M</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>+$19.05M</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>+$15.77M</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>+$15.83M</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="n">
+        <v>4182.06</v>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>88</v>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>+$14.51M</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>+$15.68M</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>RTY</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>2836.92</v>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>282</v>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>IWM</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>+$2.89M</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>+$15.19M</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="n">
-        <v>7805.11</v>
-      </c>
-      <c r="C12" s="2" t="n">
-        <v>772</v>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>+$7.54M</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>+$17.71M</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H12" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="n">
-        <v>7904.55</v>
-      </c>
-      <c r="C13" s="2" t="n">
-        <v>7845</v>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>+$16.43M</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>+$16.47M</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="n">
-        <v>4182.06</v>
-      </c>
-      <c r="C14" s="6" t="n">
-        <v>88</v>
-      </c>
-      <c r="D14" s="7" t="inlineStr">
-        <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E14" s="9" t="inlineStr">
-        <is>
-          <t>+$14.51M</t>
-        </is>
-      </c>
-      <c r="F14" s="7" t="inlineStr">
-        <is>
-          <t>+$15.68M</t>
-        </is>
-      </c>
-      <c r="G14" s="7" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H14" s="7" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+      <c r="H14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>RTY</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>2836.92</v>
+        <v>7904.55</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>282</v>
+        <v>7845</v>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>IWM</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>+$2.89M</t>
+          <t>+$14.55M</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>+$15.19M</t>
+          <t>+$14.59M</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
@@ -3535,74 +3535,74 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>RTY</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>2846.98</v>
+        <v>7799.55</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>283</v>
+        <v>7740</v>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>IWM</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="inlineStr">
-        <is>
-          <t>+$10.14M</t>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>-$5.41M</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>+$12.98M</t>
+          <t>+$13.14M</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H17" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>7799.55</v>
+        <v>2846.98</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>7740</v>
+        <v>283</v>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t>-$5.30M</t>
+          <t>IWM</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>+$10.14M</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>+$12.87M</t>
+          <t>+$12.98M</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H18" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -3623,12 +3623,12 @@
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>-$3.16M</t>
+          <t>-$3.05M</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>+$10.71M</t>
+          <t>+$10.83M</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -3789,28 +3789,28 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>7894.55</v>
+        <v>4253.35</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>7835</v>
+        <v>89.5</v>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>GDX</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>+$8.40M</t>
+          <t>+$8.23M</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>+$8.49M</t>
+          <t>+$8.35M</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
@@ -3820,107 +3820,107 @@
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>GC</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>4253.35</v>
+        <v>31095.21</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>89.5</v>
+        <v>750</v>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>GDX</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>+$8.23M</t>
+          <t>+$2.96M</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>+$8.35M</t>
+          <t>+$8.32M</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H25" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>31095.21</v>
+        <v>4277.11</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>750</v>
+        <v>90</v>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>GDX</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>+$2.96M</t>
+          <t>+$5.26M</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>+$8.32M</t>
+          <t>+$8.25M</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H26" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>GC</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>4277.11</v>
+        <v>7894.55</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>90</v>
+        <v>7835</v>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>GDX</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>+$5.26M</t>
+          <t>+$7.73M</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>+$8.25M</t>
+          <t>+$7.81M</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
@@ -3971,28 +3971,28 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>7934.55</v>
+        <v>31177.4</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>7875</v>
+        <v>752</v>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>+$6.55M</t>
+          <t>+$3.80M</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>+$6.56M</t>
+          <t>+$6.40M</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
@@ -4009,10 +4009,10 @@
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>31177.4</v>
+        <v>31506.16</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>752</v>
+        <v>760</v>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
@@ -4021,12 +4021,12 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>+$3.80M</t>
+          <t>+$4.99M</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>+$6.40M</t>
+          <t>+$5.60M</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
@@ -4039,28 +4039,28 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>31506.16</v>
+        <v>7934.55</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>760</v>
+        <v>7875</v>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>+$4.99M</t>
+          <t>+$5.36M</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>+$5.60M</t>
+          <t>+$5.37M</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">

</xml_diff>